<commit_message>
feat(fleet): align import templates with real schema + assignment columns
Drivers sheet: drop the speculative Email / Emergency Contact columns (no
matching Prisma fields) and add "Assigned Vehicle Plate". Vehicles sheet:
add "Assigned Driver Phone / Name" alongside the ICCES device ID. Banner
and info-card merges resized to the new column counts.

Guide updated to match. Templates remain a manual collection format --
no backend import endpoint exists yet.

Also updates PROGRESS.md: new "Fleet data onboarding" section, the Excel
export row for 234d191, Milestone 3.5 for the missing import endpoint/UI,
and EAS builds moved to in-progress (project linked in c99aab6).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/MERCON_Drivers_Import_Template.xlsx
+++ b/docs/templates/MERCON_Drivers_Import_Template.xlsx
@@ -759,7 +759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -769,7 +769,6 @@
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -789,8 +788,8 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>PRIMARY KEY
-Unique Phone &amp; License Number</t>
+          <t>PRIMARY KEY &amp; VEHICLE ASSIGNMENT
+Phone Number, License &amp; Assigned Vehicle Plate</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -834,12 +833,7 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Email Address</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>Emergency Contact / Notes</t>
+          <t>Assigned Vehicle Plate</t>
         </is>
       </c>
     </row>
@@ -874,14 +868,9 @@
           <t>2028-12-31</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>ahmed.mansoor@mercon.com</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Emergency: +966 55 111 2233</t>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>8492-RKA</t>
         </is>
       </c>
     </row>
@@ -916,14 +905,9 @@
           <t>2027-06-15</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>tariq.hassan@mercon.com</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="inlineStr">
-        <is>
-          <t>Heavy Truck Certified</t>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>3104-LMN</t>
         </is>
       </c>
     </row>
@@ -958,14 +942,9 @@
           <t>2029-09-20</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>john.doe@mercon.com</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>Hazmat Endorsement</t>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>9912-XYZ</t>
         </is>
       </c>
     </row>
@@ -976,8 +955,7 @@
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="14" t="n"/>
       <c r="F11" s="16" t="n"/>
-      <c r="G11" s="14" t="n"/>
-      <c r="H11" s="14" t="n"/>
+      <c r="G11" s="13" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="17" t="n"/>
@@ -986,8 +964,7 @@
       <c r="D12" s="19" t="n"/>
       <c r="E12" s="18" t="n"/>
       <c r="F12" s="20" t="n"/>
-      <c r="G12" s="18" t="n"/>
-      <c r="H12" s="18" t="n"/>
+      <c r="G12" s="17" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="13" t="n"/>
@@ -996,8 +973,7 @@
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="14" t="n"/>
       <c r="F13" s="16" t="n"/>
-      <c r="G13" s="14" t="n"/>
-      <c r="H13" s="14" t="n"/>
+      <c r="G13" s="13" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="17" t="n"/>
@@ -1006,8 +982,7 @@
       <c r="D14" s="19" t="n"/>
       <c r="E14" s="18" t="n"/>
       <c r="F14" s="20" t="n"/>
-      <c r="G14" s="18" t="n"/>
-      <c r="H14" s="18" t="n"/>
+      <c r="G14" s="17" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="13" t="n"/>
@@ -1016,8 +991,7 @@
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="14" t="n"/>
       <c r="F15" s="16" t="n"/>
-      <c r="G15" s="14" t="n"/>
-      <c r="H15" s="14" t="n"/>
+      <c r="G15" s="13" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="17" t="n"/>
@@ -1026,8 +1000,7 @@
       <c r="D16" s="19" t="n"/>
       <c r="E16" s="18" t="n"/>
       <c r="F16" s="20" t="n"/>
-      <c r="G16" s="18" t="n"/>
-      <c r="H16" s="18" t="n"/>
+      <c r="G16" s="17" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="13" t="n"/>
@@ -1036,8 +1009,7 @@
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="14" t="n"/>
       <c r="F17" s="16" t="n"/>
-      <c r="G17" s="14" t="n"/>
-      <c r="H17" s="14" t="n"/>
+      <c r="G17" s="13" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="17" t="n"/>
@@ -1046,8 +1018,7 @@
       <c r="D18" s="19" t="n"/>
       <c r="E18" s="18" t="n"/>
       <c r="F18" s="20" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="18" t="n"/>
+      <c r="G18" s="17" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="13" t="n"/>
@@ -1056,8 +1027,7 @@
       <c r="D19" s="15" t="n"/>
       <c r="E19" s="14" t="n"/>
       <c r="F19" s="16" t="n"/>
-      <c r="G19" s="14" t="n"/>
-      <c r="H19" s="14" t="n"/>
+      <c r="G19" s="13" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="17" t="n"/>
@@ -1066,8 +1036,7 @@
       <c r="D20" s="19" t="n"/>
       <c r="E20" s="18" t="n"/>
       <c r="F20" s="20" t="n"/>
-      <c r="G20" s="18" t="n"/>
-      <c r="H20" s="18" t="n"/>
+      <c r="G20" s="17" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="13" t="n"/>
@@ -1076,8 +1045,7 @@
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="14" t="n"/>
       <c r="F21" s="16" t="n"/>
-      <c r="G21" s="14" t="n"/>
-      <c r="H21" s="14" t="n"/>
+      <c r="G21" s="13" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="17" t="n"/>
@@ -1086,8 +1054,7 @@
       <c r="D22" s="19" t="n"/>
       <c r="E22" s="18" t="n"/>
       <c r="F22" s="20" t="n"/>
-      <c r="G22" s="18" t="n"/>
-      <c r="H22" s="18" t="n"/>
+      <c r="G22" s="17" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="13" t="n"/>
@@ -1096,8 +1063,7 @@
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="14" t="n"/>
       <c r="F23" s="16" t="n"/>
-      <c r="G23" s="14" t="n"/>
-      <c r="H23" s="14" t="n"/>
+      <c r="G23" s="13" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="17" t="n"/>
@@ -1106,8 +1072,7 @@
       <c r="D24" s="19" t="n"/>
       <c r="E24" s="18" t="n"/>
       <c r="F24" s="20" t="n"/>
-      <c r="G24" s="18" t="n"/>
-      <c r="H24" s="18" t="n"/>
+      <c r="G24" s="17" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="13" t="n"/>
@@ -1116,8 +1081,7 @@
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="14" t="n"/>
       <c r="F25" s="16" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
+      <c r="G25" s="13" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="17" t="n"/>
@@ -1126,8 +1090,7 @@
       <c r="D26" s="19" t="n"/>
       <c r="E26" s="18" t="n"/>
       <c r="F26" s="20" t="n"/>
-      <c r="G26" s="18" t="n"/>
-      <c r="H26" s="18" t="n"/>
+      <c r="G26" s="17" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="13" t="n"/>
@@ -1136,8 +1099,7 @@
       <c r="D27" s="15" t="n"/>
       <c r="E27" s="14" t="n"/>
       <c r="F27" s="16" t="n"/>
-      <c r="G27" s="14" t="n"/>
-      <c r="H27" s="14" t="n"/>
+      <c r="G27" s="13" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="17" t="n"/>
@@ -1146,8 +1108,7 @@
       <c r="D28" s="19" t="n"/>
       <c r="E28" s="18" t="n"/>
       <c r="F28" s="20" t="n"/>
-      <c r="G28" s="18" t="n"/>
-      <c r="H28" s="18" t="n"/>
+      <c r="G28" s="17" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="13" t="n"/>
@@ -1156,8 +1117,7 @@
       <c r="D29" s="15" t="n"/>
       <c r="E29" s="14" t="n"/>
       <c r="F29" s="16" t="n"/>
-      <c r="G29" s="14" t="n"/>
-      <c r="H29" s="14" t="n"/>
+      <c r="G29" s="13" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="17" t="n"/>
@@ -1166,8 +1126,7 @@
       <c r="D30" s="19" t="n"/>
       <c r="E30" s="18" t="n"/>
       <c r="F30" s="20" t="n"/>
-      <c r="G30" s="18" t="n"/>
-      <c r="H30" s="18" t="n"/>
+      <c r="G30" s="17" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="13" t="n"/>
@@ -1176,8 +1135,7 @@
       <c r="D31" s="15" t="n"/>
       <c r="E31" s="14" t="n"/>
       <c r="F31" s="16" t="n"/>
-      <c r="G31" s="14" t="n"/>
-      <c r="H31" s="14" t="n"/>
+      <c r="G31" s="13" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="17" t="n"/>
@@ -1186,8 +1144,7 @@
       <c r="D32" s="19" t="n"/>
       <c r="E32" s="18" t="n"/>
       <c r="F32" s="20" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="18" t="n"/>
+      <c r="G32" s="17" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="13" t="n"/>
@@ -1196,8 +1153,7 @@
       <c r="D33" s="15" t="n"/>
       <c r="E33" s="14" t="n"/>
       <c r="F33" s="16" t="n"/>
-      <c r="G33" s="14" t="n"/>
-      <c r="H33" s="14" t="n"/>
+      <c r="G33" s="13" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="17" t="n"/>
@@ -1206,8 +1162,7 @@
       <c r="D34" s="19" t="n"/>
       <c r="E34" s="18" t="n"/>
       <c r="F34" s="20" t="n"/>
-      <c r="G34" s="18" t="n"/>
-      <c r="H34" s="18" t="n"/>
+      <c r="G34" s="17" t="n"/>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="13" t="n"/>
@@ -1216,8 +1171,7 @@
       <c r="D35" s="15" t="n"/>
       <c r="E35" s="14" t="n"/>
       <c r="F35" s="16" t="n"/>
-      <c r="G35" s="14" t="n"/>
-      <c r="H35" s="14" t="n"/>
+      <c r="G35" s="13" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="17" t="n"/>
@@ -1226,8 +1180,7 @@
       <c r="D36" s="19" t="n"/>
       <c r="E36" s="18" t="n"/>
       <c r="F36" s="20" t="n"/>
-      <c r="G36" s="18" t="n"/>
-      <c r="H36" s="18" t="n"/>
+      <c r="G36" s="17" t="n"/>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="13" t="n"/>
@@ -1236,8 +1189,7 @@
       <c r="D37" s="15" t="n"/>
       <c r="E37" s="14" t="n"/>
       <c r="F37" s="16" t="n"/>
-      <c r="G37" s="14" t="n"/>
-      <c r="H37" s="14" t="n"/>
+      <c r="G37" s="13" t="n"/>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="17" t="n"/>
@@ -1246,8 +1198,7 @@
       <c r="D38" s="19" t="n"/>
       <c r="E38" s="18" t="n"/>
       <c r="F38" s="20" t="n"/>
-      <c r="G38" s="18" t="n"/>
-      <c r="H38" s="18" t="n"/>
+      <c r="G38" s="17" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="13" t="n"/>
@@ -1256,8 +1207,7 @@
       <c r="D39" s="15" t="n"/>
       <c r="E39" s="14" t="n"/>
       <c r="F39" s="16" t="n"/>
-      <c r="G39" s="14" t="n"/>
-      <c r="H39" s="14" t="n"/>
+      <c r="G39" s="13" t="n"/>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="17" t="n"/>
@@ -1266,8 +1216,7 @@
       <c r="D40" s="19" t="n"/>
       <c r="E40" s="18" t="n"/>
       <c r="F40" s="20" t="n"/>
-      <c r="G40" s="18" t="n"/>
-      <c r="H40" s="18" t="n"/>
+      <c r="G40" s="17" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="13" t="n"/>
@@ -1276,8 +1225,7 @@
       <c r="D41" s="15" t="n"/>
       <c r="E41" s="14" t="n"/>
       <c r="F41" s="16" t="n"/>
-      <c r="G41" s="14" t="n"/>
-      <c r="H41" s="14" t="n"/>
+      <c r="G41" s="13" t="n"/>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="17" t="n"/>
@@ -1286,8 +1234,7 @@
       <c r="D42" s="19" t="n"/>
       <c r="E42" s="18" t="n"/>
       <c r="F42" s="20" t="n"/>
-      <c r="G42" s="18" t="n"/>
-      <c r="H42" s="18" t="n"/>
+      <c r="G42" s="17" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="13" t="n"/>
@@ -1296,8 +1243,7 @@
       <c r="D43" s="15" t="n"/>
       <c r="E43" s="14" t="n"/>
       <c r="F43" s="16" t="n"/>
-      <c r="G43" s="14" t="n"/>
-      <c r="H43" s="14" t="n"/>
+      <c r="G43" s="13" t="n"/>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="17" t="n"/>
@@ -1306,8 +1252,7 @@
       <c r="D44" s="19" t="n"/>
       <c r="E44" s="18" t="n"/>
       <c r="F44" s="20" t="n"/>
-      <c r="G44" s="18" t="n"/>
-      <c r="H44" s="18" t="n"/>
+      <c r="G44" s="17" t="n"/>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="13" t="n"/>
@@ -1316,8 +1261,7 @@
       <c r="D45" s="15" t="n"/>
       <c r="E45" s="14" t="n"/>
       <c r="F45" s="16" t="n"/>
-      <c r="G45" s="14" t="n"/>
-      <c r="H45" s="14" t="n"/>
+      <c r="G45" s="13" t="n"/>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="17" t="n"/>
@@ -1326,8 +1270,7 @@
       <c r="D46" s="19" t="n"/>
       <c r="E46" s="18" t="n"/>
       <c r="F46" s="20" t="n"/>
-      <c r="G46" s="18" t="n"/>
-      <c r="H46" s="18" t="n"/>
+      <c r="G46" s="17" t="n"/>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="13" t="n"/>
@@ -1336,8 +1279,7 @@
       <c r="D47" s="15" t="n"/>
       <c r="E47" s="14" t="n"/>
       <c r="F47" s="16" t="n"/>
-      <c r="G47" s="14" t="n"/>
-      <c r="H47" s="14" t="n"/>
+      <c r="G47" s="13" t="n"/>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="17" t="n"/>
@@ -1346,8 +1288,7 @@
       <c r="D48" s="19" t="n"/>
       <c r="E48" s="18" t="n"/>
       <c r="F48" s="20" t="n"/>
-      <c r="G48" s="18" t="n"/>
-      <c r="H48" s="18" t="n"/>
+      <c r="G48" s="17" t="n"/>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="13" t="n"/>
@@ -1356,8 +1297,7 @@
       <c r="D49" s="15" t="n"/>
       <c r="E49" s="14" t="n"/>
       <c r="F49" s="16" t="n"/>
-      <c r="G49" s="14" t="n"/>
-      <c r="H49" s="14" t="n"/>
+      <c r="G49" s="13" t="n"/>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="17" t="n"/>
@@ -1366,8 +1306,7 @@
       <c r="D50" s="19" t="n"/>
       <c r="E50" s="18" t="n"/>
       <c r="F50" s="20" t="n"/>
-      <c r="G50" s="18" t="n"/>
-      <c r="H50" s="18" t="n"/>
+      <c r="G50" s="17" t="n"/>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="13" t="n"/>
@@ -1376,8 +1315,7 @@
       <c r="D51" s="15" t="n"/>
       <c r="E51" s="14" t="n"/>
       <c r="F51" s="16" t="n"/>
-      <c r="G51" s="14" t="n"/>
-      <c r="H51" s="14" t="n"/>
+      <c r="G51" s="13" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="17" t="n"/>
@@ -1386,8 +1324,7 @@
       <c r="D52" s="19" t="n"/>
       <c r="E52" s="18" t="n"/>
       <c r="F52" s="20" t="n"/>
-      <c r="G52" s="18" t="n"/>
-      <c r="H52" s="18" t="n"/>
+      <c r="G52" s="17" t="n"/>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="13" t="n"/>
@@ -1396,8 +1333,7 @@
       <c r="D53" s="15" t="n"/>
       <c r="E53" s="14" t="n"/>
       <c r="F53" s="16" t="n"/>
-      <c r="G53" s="14" t="n"/>
-      <c r="H53" s="14" t="n"/>
+      <c r="G53" s="13" t="n"/>
     </row>
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="17" t="n"/>
@@ -1406,8 +1342,7 @@
       <c r="D54" s="19" t="n"/>
       <c r="E54" s="18" t="n"/>
       <c r="F54" s="20" t="n"/>
-      <c r="G54" s="18" t="n"/>
-      <c r="H54" s="18" t="n"/>
+      <c r="G54" s="17" t="n"/>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="13" t="n"/>
@@ -1416,8 +1351,7 @@
       <c r="D55" s="15" t="n"/>
       <c r="E55" s="14" t="n"/>
       <c r="F55" s="16" t="n"/>
-      <c r="G55" s="14" t="n"/>
-      <c r="H55" s="14" t="n"/>
+      <c r="G55" s="13" t="n"/>
     </row>
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="17" t="n"/>
@@ -1426,8 +1360,7 @@
       <c r="D56" s="19" t="n"/>
       <c r="E56" s="18" t="n"/>
       <c r="F56" s="20" t="n"/>
-      <c r="G56" s="18" t="n"/>
-      <c r="H56" s="18" t="n"/>
+      <c r="G56" s="17" t="n"/>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="13" t="n"/>
@@ -1436,8 +1369,7 @@
       <c r="D57" s="15" t="n"/>
       <c r="E57" s="14" t="n"/>
       <c r="F57" s="16" t="n"/>
-      <c r="G57" s="14" t="n"/>
-      <c r="H57" s="14" t="n"/>
+      <c r="G57" s="13" t="n"/>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="17" t="n"/>
@@ -1446,8 +1378,7 @@
       <c r="D58" s="19" t="n"/>
       <c r="E58" s="18" t="n"/>
       <c r="F58" s="20" t="n"/>
-      <c r="G58" s="18" t="n"/>
-      <c r="H58" s="18" t="n"/>
+      <c r="G58" s="17" t="n"/>
     </row>
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="13" t="n"/>
@@ -1456,8 +1387,7 @@
       <c r="D59" s="15" t="n"/>
       <c r="E59" s="14" t="n"/>
       <c r="F59" s="16" t="n"/>
-      <c r="G59" s="14" t="n"/>
-      <c r="H59" s="14" t="n"/>
+      <c r="G59" s="13" t="n"/>
     </row>
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="17" t="n"/>
@@ -1466,15 +1396,14 @@
       <c r="D60" s="19" t="n"/>
       <c r="E60" s="18" t="n"/>
       <c r="F60" s="20" t="n"/>
-      <c r="G60" s="18" t="n"/>
-      <c r="H60" s="18" t="n"/>
+      <c r="G60" s="17" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="F4:G5"/>
     <mergeCell ref="A4:B5"/>
     <mergeCell ref="C4:E5"/>
-    <mergeCell ref="F4:H5"/>
+    <mergeCell ref="A1:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>